<commit_message>
Layout changes. Page Additions
</commit_message>
<xml_diff>
--- a/archive/Hearts_2025_26_Results_VERIFIED.xlsx
+++ b/archive/Hearts_2025_26_Results_VERIFIED.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\glorious-hearts\archive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10362F1-CCFA-404F-8457-F83CB47F214A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AE21708-995D-41F5-A103-9771510A02EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="223">
   <si>
     <t>Date</t>
   </si>
@@ -686,6 +686,12 @@
   </si>
   <si>
     <t>https://www.bbc.co.uk/sport/football/live/c0m289e39zkt</t>
+  </si>
+  <si>
+    <t>CELTIC WIN TITLE IN LAST-DAY THRILLER</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=FJdXB_damk</t>
   </si>
 </sst>
 </file>
@@ -2219,6 +2225,12 @@
       <c r="F45" s="1" t="s">
         <v>220</v>
       </c>
+      <c r="G45" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="H45" t="s">
+        <v>221</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -2310,6 +2322,7 @@
     <hyperlink ref="F44" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
     <hyperlink ref="G44" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
     <hyperlink ref="F45" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="G45" r:id="rId88" xr:uid="{F0E12E75-4B74-43B8-8F96-875B720EAA5D}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>